<commit_message>
Remove unstable SSIS project before rebuild
Removed the current SSIS project because Visual Studio/SSIS became unstable during development. Database scripts, stored procedures, views, documentation, and project structure are retained. SSIS packages will be rebuilt cleanly after the development environment is repaired.
</commit_message>
<xml_diff>
--- a/09_Source/Samples/Citi_YTD_2026.xlsx
+++ b/09_Source/Samples/Citi_YTD_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\DW_FamilyFinance\09_Source\Samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B035BC02-5D94-45EA-B1B7-4B0EA6ECE8E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D3A78AC-1765-40C7-B0B1-264EDCC66930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-915" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,18 +28,6 @@
     <t>Description</t>
   </si>
   <si>
-    <t>debit_amount</t>
-  </si>
-  <si>
-    <t>credit_amount</t>
-  </si>
-  <si>
-    <t>category</t>
-  </si>
-  <si>
-    <t>bank_name</t>
-  </si>
-  <si>
     <t>error: undefined method `first' for nil:NilClass</t>
   </si>
   <si>
@@ -77,6 +65,18 @@
   </si>
   <si>
     <t>One Drive</t>
+  </si>
+  <si>
+    <t>Credit</t>
+  </si>
+  <si>
+    <t>Debit</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>SourceName</t>
   </si>
 </sst>
 </file>
@@ -136,10 +136,10 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{EC671650-A04C-435C-AC6C-49AE5944DB24}" name="Date"/>
     <tableColumn id="2" xr3:uid="{3BB469FB-5986-4285-8515-D00FB07C19DE}" name="Description"/>
-    <tableColumn id="3" xr3:uid="{4DB2EC1A-7E9A-4650-80CC-14CE8A87941B}" name="debit_amount"/>
-    <tableColumn id="4" xr3:uid="{ACE3068D-E1D4-4E5E-9479-CAF1164A7935}" name="credit_amount"/>
-    <tableColumn id="5" xr3:uid="{52CCB14E-6A45-475F-A451-A4A385969C18}" name="category"/>
-    <tableColumn id="6" xr3:uid="{EFBD1BC9-9104-4AD2-A47A-F612E9398F40}" name="bank_name"/>
+    <tableColumn id="3" xr3:uid="{4DB2EC1A-7E9A-4650-80CC-14CE8A87941B}" name="Debit"/>
+    <tableColumn id="4" xr3:uid="{ACE3068D-E1D4-4E5E-9479-CAF1164A7935}" name="Credit"/>
+    <tableColumn id="5" xr3:uid="{52CCB14E-6A45-475F-A451-A4A385969C18}" name="Category"/>
+    <tableColumn id="6" xr3:uid="{EFBD1BC9-9104-4AD2-A47A-F612E9398F40}" name="SourceName"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -465,10 +465,10 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.75" customWidth="1"/>
-    <col min="4" max="4" width="15.375" customWidth="1"/>
+    <col min="1" max="1" width="8.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.625" customWidth="1"/>
     <col min="5" max="5" width="37.75" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.875" bestFit="1" customWidth="1"/>
   </cols>
@@ -481,16 +481,16 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -498,7 +498,7 @@
         <v>45301</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C2">
         <v>63.53</v>
@@ -507,10 +507,10 @@
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F2" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -518,7 +518,7 @@
         <v>45414</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C3">
         <v>150.57</v>
@@ -527,10 +527,10 @@
         <v>0</v>
       </c>
       <c r="E3" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -538,7 +538,7 @@
         <v>45474</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C4">
         <v>146.99</v>
@@ -547,10 +547,10 @@
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F4" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -558,7 +558,7 @@
         <v>45628</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C5">
         <v>117.96</v>
@@ -567,10 +567,10 @@
         <v>0</v>
       </c>
       <c r="E5" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F5" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -578,7 +578,7 @@
         <v>45383</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C6">
         <v>181.68</v>
@@ -587,10 +587,10 @@
         <v>0</v>
       </c>
       <c r="E6" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F6" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -598,7 +598,7 @@
         <v>45292</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C7">
         <v>195.08</v>
@@ -607,10 +607,10 @@
         <v>0</v>
       </c>
       <c r="E7" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F7" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -618,7 +618,7 @@
         <v>45476</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C8">
         <v>40.39</v>
@@ -627,10 +627,10 @@
         <v>0</v>
       </c>
       <c r="E8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F8" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -638,7 +638,7 @@
         <v>45568</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C9">
         <v>117.21</v>
@@ -647,10 +647,10 @@
         <v>0</v>
       </c>
       <c r="E9" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F9" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -658,7 +658,7 @@
         <v>45598</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C10">
         <v>136.46</v>
@@ -667,10 +667,10 @@
         <v>0</v>
       </c>
       <c r="E10" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F10" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -678,7 +678,7 @@
         <v>45352</v>
       </c>
       <c r="B11" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C11">
         <v>166.44</v>
@@ -687,10 +687,10 @@
         <v>0</v>
       </c>
       <c r="E11" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F11" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>